<commit_message>
feat: implement enrollment management system with student registration, status tracking, and transfer functionality
</commit_message>
<xml_diff>
--- a/public/templates/students_import_template.xlsx
+++ b/public/templates/students_import_template.xlsx
@@ -14,8 +14,130 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Nombres completos del estudiante (obligatorio)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Apellidos completos (obligatorio)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Formato V-12345678 o solo números (opcional)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">DD/MM/YYYY o YYYY-MM-DD (obligatorio)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">M para Masculino, F para Femenino (obligatorio)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Ej: 1er Año (opcional, para inscripción directa)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Ej: A, B, C (opcional, para inscripción directa)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
   <si>
     <t>nombres</t>
   </si>
@@ -32,46 +154,31 @@
     <t>genero</t>
   </si>
   <si>
+    <t>grado</t>
+  </si>
+  <si>
+    <t>seccion</t>
+  </si>
+  <si>
     <t>María Alejandra</t>
   </si>
   <si>
     <t>González Pérez</t>
   </si>
   <si>
-    <t>V-12345678</t>
-  </si>
-  <si>
-    <t>15/08/2010</t>
+    <t>V-34587234</t>
+  </si>
+  <si>
+    <t>15/03/2013</t>
   </si>
   <si>
     <t>F</t>
   </si>
   <si>
-    <t>INSTRUCCIONES:</t>
-  </si>
-  <si>
-    <t>• nombres: Nombres completos del estudiante. (Obligatorio)</t>
-  </si>
-  <si>
-    <t>• apellidos: Apellidos completos del estudiante. (Obligatorio)</t>
-  </si>
-  <si>
-    <t>• cedula_escolar: Formato V-12345678 o E-12345678. (Opcional — dejar vacío si no tiene)</t>
-  </si>
-  <si>
-    <t>• fecha_nacimiento: Usar formato DD/MM/YYYY. Ej: 15/08/2010. (Obligatorio)</t>
-  </si>
-  <si>
-    <t>• genero: Usar M para Masculino o F para Femenino. (Obligatorio)</t>
-  </si>
-  <si>
-    <t>• Si la cédula ya existe en el sistema, la fila se omitirá automáticamente.</t>
-  </si>
-  <si>
-    <t>• El estado del estudiante se asignará como "Regular" de forma automática.</t>
-  </si>
-  <si>
-    <t>• Eliminar las filas de instrucciones y la fila de ejemplo antes de importar.</t>
+    <t>1er Año</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -79,7 +186,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -98,35 +205,8 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="0"/>
-      <i val="1"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FF6D28D9"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FF6D28D9"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="10"/>
-      <color rgb="FF475569"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,18 +215,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6D28D9"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F3FF"/>
+        <fgColor rgb="FF336B87"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -154,50 +228,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7C3AED"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7C3AED"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7C3AED"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7C3AED"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFEDE9FE"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFEDE9FE"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFEDE9FE"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFEDE9FE"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,17 +534,19 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="true" style="0"/>
-    <col min="2" max="2" width="30" customWidth="true" style="0"/>
-    <col min="3" max="3" width="20" customWidth="true" style="0"/>
-    <col min="4" max="4" width="22" customWidth="true" style="0"/>
-    <col min="5" max="5" width="12" customWidth="true" style="0"/>
+    <col min="1" max="1" width="25" customWidth="true" style="0"/>
+    <col min="2" max="2" width="25" customWidth="true" style="0"/>
+    <col min="3" max="3" width="25" customWidth="true" style="0"/>
+    <col min="4" max="4" width="25" customWidth="true" style="0"/>
+    <col min="5" max="5" width="25" customWidth="true" style="0"/>
+    <col min="6" max="6" width="25" customWidth="true" style="0"/>
+    <col min="7" max="7" width="25" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customHeight="1" ht="24">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -523,83 +562,40 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" customHeight="1" ht="20">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="3" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="4" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="4" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="4" t="s">
+      <c r="G2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A12:E12"/>
-  </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <legacyDrawing r:id="rId_comments_vml1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add student bulk import interface with Excel template and file upload utility
</commit_message>
<xml_diff>
--- a/public/templates/students_import_template.xlsx
+++ b/public/templates/students_import_template.xlsx
@@ -14,130 +14,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">Nombres completos del estudiante (obligatorio)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">Apellidos completos (obligatorio)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">Formato V-12345678 o solo números (opcional)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">DD/MM/YYYY o YYYY-MM-DD (obligatorio)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">M para Masculino, F para Femenino (obligatorio)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">Ej: 1er Año (opcional, para inscripción directa)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">Ej: A, B, C (opcional, para inscripción directa)</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
   <si>
     <t>nombres</t>
   </si>
@@ -166,10 +44,10 @@
     <t>González Pérez</t>
   </si>
   <si>
-    <t>V-34587234</t>
-  </si>
-  <si>
-    <t>15/03/2013</t>
+    <t>V-12345678</t>
+  </si>
+  <si>
+    <t>15/08/2010</t>
   </si>
   <si>
     <t>F</t>
@@ -179,6 +57,39 @@
   </si>
   <si>
     <t>A</t>
+  </si>
+  <si>
+    <t>INSTRUCCIONES:</t>
+  </si>
+  <si>
+    <t>• nombres: Nombres completos del estudiante. (Obligatorio)</t>
+  </si>
+  <si>
+    <t>• apellidos: Apellidos completos del estudiante. (Obligatorio)</t>
+  </si>
+  <si>
+    <t>• cedula_escolar: Formato V-12345678, E-12345678 o sólo números. (Opcional — dejar vacío si no tiene)</t>
+  </si>
+  <si>
+    <t>• fecha_nacimiento: Usar formato DD/MM/YYYY o YYYY-MM-DD. Ej: 15/08/2010. (Opcional)</t>
+  </si>
+  <si>
+    <t>• genero: Usar M para Masculino o F para Femenino. (Obligatorio)</t>
+  </si>
+  <si>
+    <t>• grado: Nombre del año escolar. Ej: 1er Año, 2do Año, 3er Año. (Opcional)</t>
+  </si>
+  <si>
+    <t>• seccion: Letra de la sección. Ej: A, B. (Opcional — inscribe automáticamente en el año activo si se incluye grado)</t>
+  </si>
+  <si>
+    <t>• Si la cédula ya existe en el sistema, la fila se omitirá automáticamente.</t>
+  </si>
+  <si>
+    <t>• El estado del estudiante se asignará como "Regular" de forma automática.</t>
+  </si>
+  <si>
+    <t>• Eliminar las filas de instrucciones y la fila de ejemplo antes de importar.</t>
   </si>
 </sst>
 </file>
@@ -186,7 +97,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -205,8 +116,35 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="0"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF6D28D9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF6D28D9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="10"/>
+      <color rgb="FF475569"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -215,12 +153,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF336B87"/>
+        <fgColor rgb="FF6D28D9"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F3FF"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -228,13 +172,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7C3AED"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7C3AED"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7C3AED"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7C3AED"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFEDE9FE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFEDE9FE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFEDE9FE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFEDE9FE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,19 +515,19 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="true" style="0"/>
-    <col min="2" max="2" width="25" customWidth="true" style="0"/>
-    <col min="3" max="3" width="25" customWidth="true" style="0"/>
-    <col min="4" max="4" width="25" customWidth="true" style="0"/>
-    <col min="5" max="5" width="25" customWidth="true" style="0"/>
-    <col min="6" max="6" width="25" customWidth="true" style="0"/>
-    <col min="7" max="7" width="25" customWidth="true" style="0"/>
+    <col min="1" max="1" width="30" customWidth="true" style="0"/>
+    <col min="2" max="2" width="30" customWidth="true" style="0"/>
+    <col min="3" max="3" width="20" customWidth="true" style="0"/>
+    <col min="4" max="4" width="22" customWidth="true" style="0"/>
+    <col min="5" max="5" width="12" customWidth="true" style="0"/>
+    <col min="6" max="6" width="20" customWidth="true" style="0"/>
+    <col min="7" max="7" width="12" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" customHeight="1" ht="24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -569,33 +550,100 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
+    <row r="2" spans="1:7" customHeight="1" ht="20">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+  </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <legacyDrawing r:id="rId_comments_vml1"/>
 </worksheet>
 </file>
</xml_diff>